<commit_message>
docs(greensm-ph): finalize quotation, scope adjustments, and timeline plan
Comprehensive refinement of GreenSM Philippines project scope and estimates:

- tasks.csv: Refined DISO scope (26 tasks, 500h, $6,875) — removed contract flow,
  email templates, SMS provider tasks; reduced QA scope; added cost columns
- tasks-at.csv: Split AT/Partner scope (7 tasks, 94h, $1,531)
- summary.csv: Module breakdown with cost summary
- timeline.csv: 15-day capacity plan for 22/05/2026 deadline
- questions-for-partner.csv: Cleaned scope clarifications (4 questions, DPA focus)
- overview.md: Major restructuring (requirements → implementation → scope notes),
  login method fix (Email+Password), separate quote sections for DPA/Security/UAT
- audit-summary.md: Service-level architecture analysis and gap review
- .tmp/ audit files: Detailed service-by-service assessment
</commit_message>
<xml_diff>
--- a/gen-green/registration-grouping/sample-import-step1-initial.xlsx
+++ b/gen-green/registration-grouping/sample-import-step1-initial.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binhlt45\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vinhnguyen/workspaces/diso/accesstrade-projects/docs/gen-green/registration-grouping/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C40E9C5-4EE5-BD47-9163-F43111F01C9B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,15 +20,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -36,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="83">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -80,12 +72,6 @@
     <t>Aquafield Ocean City</t>
   </si>
   <si>
-    <t>Dịch vụ chung Vùng Nha Trang</t>
-  </si>
-  <si>
-    <t>Four Points by Sheraton Hà Giang</t>
-  </si>
-  <si>
     <t>Four Points by Sheraton Lạng Sơn</t>
   </si>
   <si>
@@ -231,33 +217,6 @@
   </si>
   <si>
     <t>HO</t>
-  </si>
-  <si>
-    <t>Match A user-cfa2cc6cd3</t>
-  </si>
-  <si>
-    <t>0977963755</t>
-  </si>
-  <si>
-    <t>Almaz</t>
-  </si>
-  <si>
-    <t>123123</t>
-  </si>
-  <si>
-    <t>00002</t>
-  </si>
-  <si>
-    <t>Match A user-51daeed94a</t>
-  </si>
-  <si>
-    <t>0977963775</t>
-  </si>
-  <si>
-    <t>VinPalace Cổ Loa</t>
-  </si>
-  <si>
-    <t>12345</t>
   </si>
   <si>
     <t>00003</t>
@@ -323,8 +282,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -340,7 +299,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -370,22 +329,22 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment vertical="center" wrapText="true"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -393,7 +352,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -406,7 +365,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -702,25 +661,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7270D39-6E24-40A3-95BE-8AC14980D531}">
-  <dimension ref="A1:M58"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:J56"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col max="2" min="1" style="1" width="9.140625"/>
-    <col customWidth="true" max="3" min="3" style="1" width="25.7109375"/>
-    <col customWidth="true" max="4" min="4" style="1" width="21"/>
-    <col customWidth="true" max="5" min="5" style="1" width="27.5703125"/>
-    <col customWidth="true" max="6" min="6" style="1" width="21.85546875"/>
-    <col max="9" min="7" style="1" width="9.140625"/>
-    <col customWidth="true" max="10" min="10" style="1" width="43.42578125"/>
-    <col max="16384" min="11" style="1" width="9.140625"/>
+    <col min="1" max="2" width="9.1640625" style="1"/>
+    <col min="3" max="3" width="25.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.83203125" style="1" customWidth="1"/>
+    <col min="7" max="9" width="9.1640625" style="1"/>
+    <col min="10" max="10" width="43.5" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
@@ -740,12 +699,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
@@ -763,382 +722,335 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="75">
+    <row r="4" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="B4" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>62</v>
-      </c>
       <c r="D4" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>68</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>28</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
-      <c r="B10" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>89</v>
-      </c>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J10" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
-      <c r="B11" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>93</v>
-      </c>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J11" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J12" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J13" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J14" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J15" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J16" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="10:10">
+    <row r="17" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J17" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="10:10">
+    <row r="18" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J18" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="10:10">
+    <row r="19" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J19" s="6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="10:10">
+    <row r="20" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J20" s="6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="10:10">
+    <row r="21" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J21" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="10:10">
+    <row r="22" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J22" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="10:10">
+    <row r="23" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J23" s="6" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="10:10">
+    <row r="24" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J24" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="10:10">
+    <row r="25" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J25" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="10:10">
+    <row r="26" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J26" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="10:10">
+    <row r="27" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J27" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="10:10">
+    <row r="28" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J28" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="10:10">
+    <row r="29" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J29" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="10:10">
+    <row r="30" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J30" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="10:10">
+    <row r="31" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J31" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="10:10">
+    <row r="32" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J32" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="10:10">
+    <row r="33" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J33" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="10:10">
+    <row r="34" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J34" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="10:10">
+    <row r="35" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J35" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="36" spans="10:10">
+    <row r="36" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J36" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="10:10">
+    <row r="37" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J37" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="10:10">
+    <row r="38" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J38" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="10:10">
+    <row r="39" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J39" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="10:10">
+    <row r="40" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J40" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="10:10">
+    <row r="41" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J41" s="6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="10:10">
+    <row r="42" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J42" s="6" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="43" spans="10:10">
+    <row r="43" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J43" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="44" spans="10:10">
+    <row r="44" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J44" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J45" s="6" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="45" spans="10:10">
-      <c r="J45" s="6" t="s">
+    <row r="46" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J46" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="46" spans="10:10">
-      <c r="J46" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="47" spans="10:10">
+    <row r="47" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J47" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="48" spans="10:10">
-      <c r="J48" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="49" spans="10:10">
-      <c r="J49" s="6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="50" spans="10:10">
-      <c r="J50" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55" spans="10:10">
+    <row r="48" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J48" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="53" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J53" s="6"/>
+    </row>
+    <row r="54" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J54" s="6"/>
+    </row>
+    <row r="55" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J55" s="6"/>
     </row>
-    <row r="56" spans="10:10">
+    <row r="56" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J56" s="6"/>
-    </row>
-    <row r="57" spans="10:10">
-      <c r="J57" s="6"/>
-    </row>
-    <row r="58" spans="10:10">
-      <c r="J58" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup r:id="rId1" orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>